<commit_message>
Exploratory Data Analysis - TF-IDF Analysis
</commit_message>
<xml_diff>
--- a/outputs/data_dictionary_initial.xlsx
+++ b/outputs/data_dictionary_initial.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -463,7 +463,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Customer review text</t>
+          <t>Categories of products being reviewed</t>
         </is>
       </c>
     </row>
@@ -480,7 +480,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Customer rating</t>
+          <t>Date and time review was submitted</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Product category</t>
+          <t>Customer rating</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sentiment label</t>
+          <t>Customer review text</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Date and time review was submitted</t>
+          <t>Sentiment label</t>
         </is>
       </c>
     </row>

</xml_diff>